<commit_message>
Auto update Pengadaan 2026-08-26 14:59:06
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-26).xlsx
@@ -2777,22 +2777,22 @@
         <v>354293991</v>
       </c>
       <c r="E64" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>129198291</v>
+        <v>115323291</v>
       </c>
       <c r="G64" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H64" s="10" t="n">
-        <v>127533150</v>
+        <v>113833150</v>
       </c>
       <c r="I64" s="8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J64" s="10" t="n">
-        <v>225095700</v>
+        <v>238970700</v>
       </c>
     </row>
     <row r="65" ht="45" customHeight="1">
@@ -2877,22 +2877,22 @@
         <v>32463190559</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>5678297657</v>
+        <v>5664422657</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>5194303674</v>
+        <v>5180603674</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3565</v>
+        <v>3567</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>26784892902</v>
+        <v>26798767902</v>
       </c>
     </row>
   </sheetData>
@@ -3670,34 +3670,38 @@
         <v>1109929988</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>873381088</v>
+        <v>817625000</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>870460930</v>
+        <v>814796650</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>870460930</v>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>55664280</v>
+        <v>814796650</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="10" t="n">
-        <v>236548900</v>
+        <v>292304988</v>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
@@ -3716,34 +3720,38 @@
         <v>1888168641</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1162285000</v>
+        <v>966980500</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1157390640</v>
+        <v>962557890</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>900653190</v>
-      </c>
-      <c r="K19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>194832750</v>
+        <v>705820440</v>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M19" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>725883641</v>
+        <v>921188141</v>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -6414,34 +6422,34 @@
         <v>94872478306</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>58216182104</v>
+        <v>57965121516</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>55737866422.43</v>
+        <v>55487369392.43</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>27428763177</v>
+        <v>27178266147</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L67" s="13" t="n">
-        <v>764123653</v>
+        <v>513626623</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>36656296202</v>
+        <v>36907356790</v>
       </c>
     </row>
   </sheetData>
@@ -8167,38 +8175,38 @@
         <v>520638000</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>520638000</v>
+        <v>243138000</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>514867950</v>
+        <v>243123300</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>514867950</v>
-      </c>
-      <c r="K34" s="8" t="n">
+        <v>243123300</v>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="L34" s="10" t="n">
-        <v>271744650</v>
-      </c>
-      <c r="M34" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N34" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N34" s="10" t="n">
+        <v>277500000</v>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
@@ -10291,34 +10299,34 @@
         <v>173330864188</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>131577396506</v>
+        <v>131299896506</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>64463346946.01</v>
+        <v>64191602296.01</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>60644763146</v>
+        <v>60373018496</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L67" s="13" t="n">
-        <v>2980144727</v>
+        <v>2708400077</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>41753467682</v>
+        <v>42030967682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>